<commit_message>
batch 1408 v2: recover 2 dropped rows (Banochka, Legion VI) -> 231/231; regenerated stitches, part1, xlsx, manifest
</commit_message>
<xml_diff>
--- a/1408/members_14_08_2026_part1.xlsx
+++ b/1408/members_14_08_2026_part1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="248">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -764,6 +764,12 @@
     <t xml:space="preserve">Legion II</t>
   </si>
   <si>
+    <t xml:space="preserve">Баночка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legion VI</t>
+  </si>
+  <si>
     <t xml:space="preserve">Legion VII</t>
   </si>
   <si>
@@ -797,31 +803,40 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Source video: Viking_Rise_2026-08-15_06-46-33.mp4 (uploaded 2026-08-15). Capture date: 2026-08-14 (per user; NOT re-confirmed).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resolution 1328x748. 249 frames @1fps. Row detection: per-row binary-mask XOR mutual-best matching + global clustering.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rows read: 229 of 229 detected. No unbridged seam, no [hidden], no [unread]. Power strictly decreasing; no duplicate (Power,KP,ActPts) triples.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambiguous all-vertical-stroke names written as I x N with [strokes=N]; stroke counts stable over 3 frames and thresholds 120/140/150.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  row 116 strokes=13 | row 169 strokes=11 | row 173 strokes=10 | row 185 strokes=15 (first stem is a taller L, not avatar edge) | row 189 strokes=11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identity for these rows must come from Power + Kill Points + Activity Points, never from stroke count.</t>
+    <t xml:space="preserve">Source video: Viking_Rise_2026-08-15_06-46-33.mp4 (uploaded 2026-08-15). Capture date: 2026-08-14 (per user).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolution 1328x748. 249 frames @1fps. Row detection: per-row binary-mask XOR mutual-best matching -&gt; union-find row identity -&gt; global-position clustering.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rows read: 231 of 231. Matches the member count Ha read on the game UI. No [hidden], no [unread], no unbridged seam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power strictly decreasing across all 231 rows; no duplicate (Power, Kill Points, Activity Points) triple.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORRECTION vs first pass: the first pass reported 229 rows. Scroll measurement was wrong by ~2 row pitches at frames 0231-0234 (in-game popup broke the mask alignment), folding 2 rows into their neighbours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Recovered by visual re-inspection of frames 0230/0231/0232/0233/0234/0238: row 220 Baнoчka and row 221 Legion VI, both between Legion II and Legion VII.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Frames 0106 and 0108 also had wrong dy (-82 / +85, true 0 / 0) but the errors cancelled - no row lost there; verified visually (l3omb -&gt; skywraiith -&gt; UHTRED BR contiguous).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambiguous all-vertical-stroke names written as I x N with [strokes=N]; counts stable over 3 frames and thresholds 120/140/150.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  row 116 strokes=13 | row 169 strokes=11 | row 173 strokes=10 | row 185 strokes=15 (first stem is a taller L, not the avatar edge) | row 189 strokes=11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rows 169 and 189 carry the SAME stroke count (11) but are different members - match by Power + Kill Points + Activity Points only, never by name string.</t>
   </si>
   <si>
     <t xml:space="preserve">Row 132 (hab1st) was the highlighted/selected row on screen (blue background) - read normally.</t>
   </si>
   <si>
     <t xml:space="preserve">Row 133 (Herooo) Activity Points = 0 as displayed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expected member count from game UI: NOT YET PROVIDED by user - 229 is a measured number only.</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1254,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E241"/>
+  <dimension ref="A1:E246"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -4996,13 +5011,13 @@
         <v>223</v>
       </c>
       <c r="C221" s="5" t="n">
-        <v>81585311</v>
+        <v>85129509</v>
       </c>
       <c r="D221" s="5" t="n">
-        <v>158051518</v>
+        <v>110779611</v>
       </c>
       <c r="E221" s="5" t="n">
-        <v>3469100</v>
+        <v>16596433</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5013,13 +5028,13 @@
         <v>224</v>
       </c>
       <c r="C222" s="3" t="n">
-        <v>68084500</v>
+        <v>83506540</v>
       </c>
       <c r="D222" s="3" t="n">
-        <v>96685162</v>
+        <v>197238323</v>
       </c>
       <c r="E222" s="3" t="n">
-        <v>7105072</v>
+        <v>6951490</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5030,13 +5045,13 @@
         <v>225</v>
       </c>
       <c r="C223" s="5" t="n">
-        <v>65796486</v>
+        <v>81585311</v>
       </c>
       <c r="D223" s="5" t="n">
-        <v>61408972</v>
+        <v>158051518</v>
       </c>
       <c r="E223" s="5" t="n">
-        <v>6269311</v>
+        <v>3469100</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5047,13 +5062,13 @@
         <v>226</v>
       </c>
       <c r="C224" s="3" t="n">
-        <v>64335398</v>
+        <v>68084500</v>
       </c>
       <c r="D224" s="3" t="n">
-        <v>71505002</v>
+        <v>96685162</v>
       </c>
       <c r="E224" s="3" t="n">
-        <v>7048346</v>
+        <v>7105072</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5064,13 +5079,13 @@
         <v>227</v>
       </c>
       <c r="C225" s="5" t="n">
-        <v>56548233</v>
+        <v>65796486</v>
       </c>
       <c r="D225" s="5" t="n">
-        <v>97267069</v>
+        <v>61408972</v>
       </c>
       <c r="E225" s="5" t="n">
-        <v>6750535</v>
+        <v>6269311</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5081,13 +5096,13 @@
         <v>228</v>
       </c>
       <c r="C226" s="3" t="n">
-        <v>56179771</v>
+        <v>64335398</v>
       </c>
       <c r="D226" s="3" t="n">
-        <v>54092935</v>
+        <v>71505002</v>
       </c>
       <c r="E226" s="3" t="n">
-        <v>6493439</v>
+        <v>7048346</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5098,13 +5113,13 @@
         <v>229</v>
       </c>
       <c r="C227" s="5" t="n">
-        <v>53898602</v>
+        <v>56548233</v>
       </c>
       <c r="D227" s="5" t="n">
-        <v>95368497</v>
+        <v>97267069</v>
       </c>
       <c r="E227" s="5" t="n">
-        <v>6016415</v>
+        <v>6750535</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5115,13 +5130,13 @@
         <v>230</v>
       </c>
       <c r="C228" s="3" t="n">
-        <v>49749161</v>
+        <v>56179771</v>
       </c>
       <c r="D228" s="3" t="n">
-        <v>162374326</v>
+        <v>54092935</v>
       </c>
       <c r="E228" s="3" t="n">
-        <v>6876612</v>
+        <v>6493439</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5132,13 +5147,13 @@
         <v>231</v>
       </c>
       <c r="C229" s="5" t="n">
-        <v>43454468</v>
+        <v>53898602</v>
       </c>
       <c r="D229" s="5" t="n">
-        <v>25976835</v>
+        <v>95368497</v>
       </c>
       <c r="E229" s="5" t="n">
-        <v>2971700</v>
+        <v>6016415</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5149,40 +5164,64 @@
         <v>232</v>
       </c>
       <c r="C230" s="3" t="n">
+        <v>49749161</v>
+      </c>
+      <c r="D230" s="3" t="n">
+        <v>162374326</v>
+      </c>
+      <c r="E230" s="3" t="n">
+        <v>6876612</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="4" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C231" s="5" t="n">
+        <v>43454468</v>
+      </c>
+      <c r="D231" s="5" t="n">
+        <v>25976835</v>
+      </c>
+      <c r="E231" s="5" t="n">
+        <v>2971700</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C232" s="3" t="n">
         <v>22532681</v>
       </c>
-      <c r="D230" s="3" t="n">
+      <c r="D232" s="3" t="n">
         <v>117384</v>
       </c>
-      <c r="E230" s="3" t="n">
+      <c r="E232" s="3" t="n">
         <v>676427</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B231" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="C231" s="8" t="n">
-        <f aca="false">SUM(C2:C230)</f>
-        <v>37867867026</v>
-      </c>
-      <c r="D231" s="8" t="n">
-        <f aca="false">SUM(D2:D230)</f>
-        <v>972668563782</v>
-      </c>
-      <c r="E231" s="8" t="n">
-        <f aca="false">SUM(E2:E230)</f>
-        <v>3983434906</v>
-      </c>
-    </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B233" s="9" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B234" s="9" t="s">
+      <c r="B233" s="7" t="s">
         <v>235</v>
+      </c>
+      <c r="C233" s="8" t="n">
+        <f aca="false">SUM(C2:C232)</f>
+        <v>38036503075</v>
+      </c>
+      <c r="D233" s="8" t="n">
+        <f aca="false">SUM(D2:D232)</f>
+        <v>972976581716</v>
+      </c>
+      <c r="E233" s="8" t="n">
+        <f aca="false">SUM(E2:E232)</f>
+        <v>4006982829</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5218,6 +5257,31 @@
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B241" s="9" t="s">
         <v>242</v>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B242" s="9" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B243" s="9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B244" s="9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B245" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B246" s="9" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>